<commit_message>
Final outputs for paper
</commit_message>
<xml_diff>
--- a/model/Output_Budget/1. Baseline/Grid Search/Evaluation Metrics.xlsx
+++ b/model/Output_Budget/1. Baseline/Grid Search/Evaluation Metrics.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>2000000</t>
+          <t>1250000</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -473,19 +473,19 @@
         <v>0.29</v>
       </c>
       <c r="D2" t="n">
-        <v>0.03803033241160274</v>
+        <v>0.03798457210800329</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1688275074800518</v>
+        <v>0.1680424388600761</v>
       </c>
       <c r="F2" t="n">
-        <v>9733359.33101703</v>
+        <v>9734124.342999995</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1250000</t>
+          <t>1500000</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -495,167 +495,167 @@
         <v>0.29</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03800595928583105</v>
+        <v>0.03798457210800329</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1690402211659043</v>
+        <v>0.168042438860076</v>
       </c>
       <c r="F3" t="n">
-        <v>9733525.556279989</v>
+        <v>9734124.342999995</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>1500000</t>
+          <t>250000</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04</v>
+        <v>0.13</v>
       </c>
       <c r="C4" t="n">
-        <v>0.29</v>
+        <v>0.37</v>
       </c>
       <c r="D4" t="n">
-        <v>0.03800595928583131</v>
+        <v>0.1449055985710506</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1690402211659048</v>
+        <v>0.1291650720003819</v>
       </c>
       <c r="F4" t="n">
-        <v>9733525.556279989</v>
+        <v>7926212.885027498</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>1750000</t>
+          <t>100000</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04</v>
+        <v>0.13</v>
       </c>
       <c r="C5" t="n">
-        <v>0.29</v>
+        <v>0.4</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03800595928582916</v>
+        <v>0.3583682720485077</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1689550632530328</v>
+        <v>0.2234802810223456</v>
       </c>
       <c r="F5" t="n">
-        <v>9733570.579604594</v>
+        <v>5700859.529451682</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>1000000</t>
+          <t>2000000</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="D6" t="n">
-        <v>0.03800595928583134</v>
+        <v>0.03798457210800325</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1751000135766082</v>
+        <v>0.168042438860076</v>
       </c>
       <c r="F6" t="n">
-        <v>9674468.732703272</v>
+        <v>9734124.342999993</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>100000</t>
+          <t>400000</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3579565362877447</v>
+        <v>0.1390739428283676</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2234905246335453</v>
+        <v>0.09207941150463429</v>
       </c>
       <c r="F7" t="n">
-        <v>5702040.299289487</v>
+        <v>8258752.379616951</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>250000</t>
+          <t>1750000</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.13</v>
+        <v>0.04</v>
       </c>
       <c r="C8" t="n">
-        <v>0.37</v>
+        <v>0.29</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1450165554679115</v>
+        <v>0.03798457210800329</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1292631618042654</v>
+        <v>0.1680424388600759</v>
       </c>
       <c r="F8" t="n">
-        <v>7925329.901743376</v>
+        <v>9734124.342999997</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>750000</t>
+          <t>1000000</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="C9" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02881462013567902</v>
+        <v>0.03798457210800332</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1017485083098398</v>
+        <v>0.1741155494467129</v>
       </c>
       <c r="F9" t="n">
-        <v>9520723.85954579</v>
+        <v>9675252.004419912</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>400000</t>
+          <t>750000</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1242550698143148</v>
+        <v>0.02695802279162152</v>
       </c>
       <c r="E10" t="n">
-        <v>0.09791687318987</v>
+        <v>0.0971584969000366</v>
       </c>
       <c r="F10" t="n">
-        <v>8360817.78629115</v>
+        <v>9446392.038026927</v>
       </c>
     </row>
   </sheetData>

</xml_diff>